<commit_message>
Fix basket target, dynamic level checks, and cascade safety validations
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step.xlsx
@@ -772,15 +772,13 @@
           <t>No opposite cascade active</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+      <c r="B6">
+        <f>IF(AND(SectionCalculator_UP!B2="SELL",COUNTIFS(CurrentPositions!B2:B500,"BUY",CurrentPositions!C2:C500,"SECTION_BIG")=0),"OK",IF(SectionCalculator_UP!B2&lt;&gt;"SELL","OK","ERROR"))</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>IF(AND(SectionCalculator_DOWN!B2="BUY",COUNTIFS(CurrentPositions!B2:B500,"SELL",CurrentPositions!C2:C500,"SECTION_BIG")=0),"OK",IF(SectionCalculator_DOWN!B2&lt;&gt;"BUY","OK","ERROR"))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -18430,7 +18428,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>ABS(SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"BUY")-SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"SELL"))</f>
+        <f>ABS(SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"BUY")+IF(B2="BUY",B7,0)+IF(B2="SELL",B8,0)-SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"SELL")-IF(B2="SELL",B7,0)-IF(B2="BUY",B8,0))</f>
         <v/>
       </c>
     </row>
@@ -18441,7 +18439,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>IF(Scenario_UP!B4&gt;=Scenario_UP!E4,"YES","NO")</f>
+        <f>IF(Scenario_UP!B4&gt;=INDEX(Scenario_UP!E4:E7,B4),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -18951,7 +18949,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>ABS(SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"BUY")-SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"SELL"))</f>
+        <f>ABS(SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"BUY")+IF(B2="BUY",B7,0)+IF(B2="SELL",B8,0)-SUMIFS(CurrentPositions!D2:D500,CurrentPositions!B2:B500,"SELL")-IF(B2="SELL",B7,0)-IF(B2="BUY",B8,0))</f>
         <v/>
       </c>
     </row>
@@ -18962,7 +18960,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>IF(Scenario_DOWN!B4&lt;=Scenario_DOWN!E9,"YES","NO")</f>
+        <f>IF(Scenario_DOWN!B4&lt;=INDEX(Scenario_DOWN!E9:E12,B4),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19881,11 +19879,11 @@
         </is>
       </c>
       <c r="B10">
-        <f>IF(B3+B4&gt;=Settings!$B$10,"YES","NO")</f>
+        <f>IF(B3+B4&gt;=Settings!$B$11,"YES","NO")</f>
         <v/>
       </c>
       <c r="C10">
-        <f>IF(C3+C4&gt;=Settings!$B$10,"YES","NO")</f>
+        <f>IF(C3+C4&gt;=Settings!$B$11,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize recovery-lock workbook generator and remove legacy artifacts
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step.xlsx
@@ -614,6 +614,18 @@
         <v>0</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CostMode</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FULL_CYCLE</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
@@ -686,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -758,11 +770,11 @@
         </is>
       </c>
       <c r="B5">
-        <f>IF(OR(SectionCalculator_UP!B13="NO",SectionCalculator_UP!B12="YES"),"OK","ERROR")</f>
+        <f>IF(OR(SectionCalculator_UP!B14="NO",SectionCalculator_UP!B12="YES"),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C5">
-        <f>IF(OR(SectionCalculator_DOWN!B13="NO",SectionCalculator_DOWN!B12="YES"),"OK","ERROR")</f>
+        <f>IF(OR(SectionCalculator_DOWN!B14="NO",SectionCalculator_DOWN!B12="YES"),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
@@ -773,41 +785,11 @@
         </is>
       </c>
       <c r="B6">
-        <f>IF(AND(SectionCalculator_UP!B2="SELL",COUNTIFS(CurrentPositions!B2:B500,"BUY",CurrentPositions!C2:C500,"SECTION_BIG")=0),"OK",IF(SectionCalculator_UP!B2&lt;&gt;"SELL","OK","ERROR"))</f>
+        <f>IF(SectionCalculator_UP!B13="YES","OK","ERROR")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>IF(AND(SectionCalculator_DOWN!B2="BUY",COUNTIFS(CurrentPositions!B2:B500,"SELL",CurrentPositions!C2:C500,"SECTION_BIG")=0),"OK",IF(SectionCalculator_DOWN!B2&lt;&gt;"BUY","OK","ERROR"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CloseLot &lt; MinLot =&gt; do not close</t>
-        </is>
-      </c>
-      <c r="B7">
-        <f>IF(OR(TailRecovery_UP!B10&gt;=Settings!$B$6,TailRecovery_UP!B10=0),"OK","ERROR")</f>
-        <v/>
-      </c>
-      <c r="C7">
-        <f>IF(OR(TailRecovery_DOWN!B10&gt;=Settings!$B$6,TailRecovery_DOWN!B10=0),"OK","ERROR")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>RecoveryFundAfterClose &gt;= 0</t>
-        </is>
-      </c>
-      <c r="B8">
-        <f>IF(TailRecovery_UP!B13&gt;=0,"OK","ERROR")</f>
-        <v/>
-      </c>
-      <c r="C8">
-        <f>IF(TailRecovery_DOWN!B13&gt;=0,"OK","ERROR")</f>
+        <f>IF(SectionCalculator_DOWN!B13="YES","OK","ERROR")</f>
         <v/>
       </c>
     </row>
@@ -822,18 +804,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>"NEXT ACTION UP:"&amp;CHAR(10)&amp;"CloseSection="&amp;BasketSummary!B8&amp;CHAR(10)&amp;"CloseTail="&amp;BasketSummary!B9&amp;CHAR(10)&amp;"CloseLot="&amp;TEXT(BasketSummary!B7,"0.00")&amp;CHAR(10)&amp;"TailAfter="&amp;TEXT(BasketSummary!B6,"0.00")&amp;CHAR(10)&amp;"NextSection Big/Small="&amp;TEXT(BasketSummary!B11,"0.00")&amp;"/"&amp;TEXT(BasketSummary!B12,"0.00")&amp;CHAR(10)&amp;"Action="&amp;BasketSummary!B13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <f>"NEXT ACTION DOWN:"&amp;CHAR(10)&amp;"CloseSection="&amp;BasketSummary!C8&amp;CHAR(10)&amp;"CloseTail="&amp;BasketSummary!C9&amp;CHAR(10)&amp;"CloseLot="&amp;TEXT(BasketSummary!C7,"0.00")&amp;CHAR(10)&amp;"TailAfter="&amp;TEXT(BasketSummary!C6,"0.00")&amp;CHAR(10)&amp;"NextSection Big/Small="&amp;TEXT(BasketSummary!C11,"0.00")&amp;"/"&amp;TEXT(BasketSummary!C12,"0.00")&amp;CHAR(10)&amp;"Action="&amp;BasketSummary!C13</f>
+        <f>"NEXT ACTION UP:"&amp;CHAR(10)&amp;BasketSummary!B13&amp;CHAR(10)&amp;"NEXT ACTION DOWN:"&amp;CHAR(10)&amp;BasketSummary!C13</f>
         <v/>
       </c>
     </row>
@@ -1074,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J224"/>
+  <dimension ref="A1:J225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9639,44 +9615,55 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>TailTicket</t>
+          <t>TailWorstPnL</t>
         </is>
       </c>
       <c r="B221">
-        <f>IFERROR(INDEX(A7:A206,MATCH(MINIFS(H7:H206,B7:B206,"SELL",H7:H206,"&lt;0"),H7:H206,0)),"N/A")</f>
+        <f>MINIFS(H7:H206,B7:B206,"SELL",H7:H206,"&lt;0")</f>
         <v/>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>TailLot</t>
+          <t>TailTicket</t>
         </is>
       </c>
       <c r="B222">
-        <f>IF(B221="N/A",0,XLOOKUP(B221,A7:A206,D7:D206,0))</f>
+        <f>IFERROR(MINIFS(A7:A206,B7:B206,"SELL",H7:H206,B221),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>TailLossMoney</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B223">
-        <f>IF(B221="N/A",0,ABS(XLOOKUP(B221,A7:A206,H7:H206,0)))</f>
+        <f>IF(B222="N/A",0,XLOOKUP(B222,A7:A206,D7:D206,0))</f>
         <v/>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
+          <t>TailLossMoney</t>
+        </is>
+      </c>
+      <c r="B224">
+        <f>IF(B222="N/A",0,ABS(XLOOKUP(B222,A7:A206,H7:H206,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
           <t>TailLossPerLot</t>
         </is>
       </c>
-      <c r="B224">
-        <f>IF(B222=0,0,ABS(B223/B222))</f>
+      <c r="B225">
+        <f>IF(B223=0,0,ABS(B224/B223))</f>
         <v/>
       </c>
     </row>
@@ -9691,7 +9678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J224"/>
+  <dimension ref="A1:J225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18256,44 +18243,55 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>TailTicket</t>
+          <t>TailWorstPnL</t>
         </is>
       </c>
       <c r="B221">
-        <f>IFERROR(INDEX(A7:A206,MATCH(MINIFS(H7:H206,B7:B206,"BUY",H7:H206,"&lt;0"),H7:H206,0)),"N/A")</f>
+        <f>MINIFS(H7:H206,B7:B206,"BUY",H7:H206,"&lt;0")</f>
         <v/>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>TailLot</t>
+          <t>TailTicket</t>
         </is>
       </c>
       <c r="B222">
-        <f>IF(B221="N/A",0,XLOOKUP(B221,A7:A206,D7:D206,0))</f>
+        <f>IFERROR(MINIFS(A7:A206,B7:B206,"BUY",H7:H206,B221),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>TailLossMoney</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B223">
-        <f>IF(B221="N/A",0,ABS(XLOOKUP(B221,A7:A206,H7:H206,0)))</f>
+        <f>IF(B222="N/A",0,XLOOKUP(B222,A7:A206,D7:D206,0))</f>
         <v/>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
+          <t>TailLossMoney</t>
+        </is>
+      </c>
+      <c r="B224">
+        <f>IF(B222="N/A",0,ABS(XLOOKUP(B222,A7:A206,H7:H206,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
           <t>TailLossPerLot</t>
         </is>
       </c>
-      <c r="B224">
-        <f>IF(B222=0,0,ABS(B223/B222))</f>
+      <c r="B225">
+        <f>IF(B223=0,0,ABS(B224/B223))</f>
         <v/>
       </c>
     </row>
@@ -18341,7 +18339,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>Scenario_UP!B222</f>
+        <f>Scenario_UP!B223</f>
         <v/>
       </c>
     </row>
@@ -18446,11 +18444,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>NoOppositeCascade</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>IF(B2="SELL",IF(COUNTIFS(CurrentPositions!B2:B500,"BUY",CurrentPositions!C2:C500,"SECTION_BIG")=0,"YES","NO"),IF(B2="BUY",IF(COUNTIFS(CurrentPositions!B2:B500,"SELL",CurrentPositions!C2:C500,"SECTION_BIG")=0,"YES","NO"),"NO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>CanOpenSection</t>
         </is>
       </c>
-      <c r="B13">
-        <f>IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES"),"YES","NO")</f>
+      <c r="B14">
+        <f>IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES",B13="YES"),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -18564,7 +18573,7 @@
         <v/>
       </c>
       <c r="K21">
-        <f>(Settings!$B$12*Settings!$B$4*(C21+F21))+(Settings!$B$13*(C21+F21))+(Settings!$B$14*(C21+F21))</f>
+        <f>LET(Lots,C21+F21,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L21">
@@ -18619,7 +18628,7 @@
         <v/>
       </c>
       <c r="K22">
-        <f>(Settings!$B$12*Settings!$B$4*(C22+F22))+(Settings!$B$13*(C22+F22))+(Settings!$B$14*(C22+F22))</f>
+        <f>LET(Lots,C22+F22,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L22">
@@ -18674,7 +18683,7 @@
         <v/>
       </c>
       <c r="K23">
-        <f>(Settings!$B$12*Settings!$B$4*(C23+F23))+(Settings!$B$13*(C23+F23))+(Settings!$B$14*(C23+F23))</f>
+        <f>LET(Lots,C23+F23,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L23">
@@ -18729,7 +18738,7 @@
         <v/>
       </c>
       <c r="K24">
-        <f>(Settings!$B$12*Settings!$B$4*(C24+F24))+(Settings!$B$13*(C24+F24))+(Settings!$B$14*(C24+F24))</f>
+        <f>LET(Lots,C24+F24,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L24">
@@ -18862,7 +18871,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>Scenario_DOWN!B222</f>
+        <f>Scenario_DOWN!B223</f>
         <v/>
       </c>
     </row>
@@ -18967,11 +18976,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>NoOppositeCascade</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>IF(B2="SELL",IF(COUNTIFS(CurrentPositions!B2:B500,"BUY",CurrentPositions!C2:C500,"SECTION_BIG")=0,"YES","NO"),IF(B2="BUY",IF(COUNTIFS(CurrentPositions!B2:B500,"SELL",CurrentPositions!C2:C500,"SECTION_BIG")=0,"YES","NO"),"NO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>CanOpenSection</t>
         </is>
       </c>
-      <c r="B13">
-        <f>IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES"),"YES","NO")</f>
+      <c r="B14">
+        <f>IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES",B13="YES"),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19085,7 +19105,7 @@
         <v/>
       </c>
       <c r="K21">
-        <f>(Settings!$B$12*Settings!$B$4*(C21+F21))+(Settings!$B$13*(C21+F21))+(Settings!$B$14*(C21+F21))</f>
+        <f>LET(Lots,C21+F21,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L21">
@@ -19140,7 +19160,7 @@
         <v/>
       </c>
       <c r="K22">
-        <f>(Settings!$B$12*Settings!$B$4*(C22+F22))+(Settings!$B$13*(C22+F22))+(Settings!$B$14*(C22+F22))</f>
+        <f>LET(Lots,C22+F22,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L22">
@@ -19195,7 +19215,7 @@
         <v/>
       </c>
       <c r="K23">
-        <f>(Settings!$B$12*Settings!$B$4*(C23+F23))+(Settings!$B$13*(C23+F23))+(Settings!$B$14*(C23+F23))</f>
+        <f>LET(Lots,C23+F23,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L23">
@@ -19250,7 +19270,7 @@
         <v/>
       </c>
       <c r="K24">
-        <f>(Settings!$B$12*Settings!$B$4*(C24+F24))+(Settings!$B$13*(C24+F24))+(Settings!$B$14*(C24+F24))</f>
+        <f>LET(Lots,C24+F24,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
         <v/>
       </c>
       <c r="L24">
@@ -19350,7 +19370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19383,7 +19403,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>Scenario_UP!B221</f>
+        <f>Scenario_UP!B222</f>
         <v/>
       </c>
     </row>
@@ -19394,7 +19414,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>Scenario_UP!B222</f>
+        <f>Scenario_UP!B223</f>
         <v/>
       </c>
     </row>
@@ -19405,7 +19425,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>Scenario_UP!B224</f>
+        <f>Scenario_UP!B225</f>
         <v/>
       </c>
     </row>
@@ -19511,22 +19531,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NextBigLotAfterRecovery</t>
+          <t>NextLevel</t>
         </is>
       </c>
       <c r="B15">
-        <f>FLOOR(B14*XLOOKUP(1,Settings!A21:A24,Settings!B21:B24),Settings!$B$7)</f>
+        <f>SectionCalculator_UP!B4</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>NextBigLotAfterRecovery</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!B21:B24),Settings!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>NextSmallLotAfterRecovery</t>
         </is>
       </c>
-      <c r="B16">
-        <f>FLOOR(B14*XLOOKUP(1,Settings!A21:A24,Settings!C21:C24),Settings!$B$7)</f>
+      <c r="B17">
+        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!C21:C24),Settings!$B$7)</f>
         <v/>
       </c>
     </row>
@@ -19541,7 +19572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19574,7 +19605,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>Scenario_DOWN!B221</f>
+        <f>Scenario_DOWN!B222</f>
         <v/>
       </c>
     </row>
@@ -19585,7 +19616,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>Scenario_DOWN!B222</f>
+        <f>Scenario_DOWN!B223</f>
         <v/>
       </c>
     </row>
@@ -19596,7 +19627,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>Scenario_DOWN!B224</f>
+        <f>Scenario_DOWN!B225</f>
         <v/>
       </c>
     </row>
@@ -19702,22 +19733,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NextBigLotAfterRecovery</t>
+          <t>NextLevel</t>
         </is>
       </c>
       <c r="B15">
-        <f>FLOOR(B14*XLOOKUP(1,Settings!A21:A24,Settings!B21:B24),Settings!$B$7)</f>
+        <f>SectionCalculator_DOWN!B4</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>NextBigLotAfterRecovery</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!B21:B24),Settings!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>NextSmallLotAfterRecovery</t>
         </is>
       </c>
-      <c r="B16">
-        <f>FLOOR(B14*XLOOKUP(1,Settings!A21:A24,Settings!C21:C24),Settings!$B$7)</f>
+      <c r="B17">
+        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!C21:C24),Settings!$B$7)</f>
         <v/>
       </c>
     </row>
@@ -19894,11 +19936,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>TailRecovery_UP!B15</f>
+        <f>TailRecovery_UP!B16</f>
         <v/>
       </c>
       <c r="C11">
-        <f>TailRecovery_DOWN!B15</f>
+        <f>TailRecovery_DOWN!B16</f>
         <v/>
       </c>
     </row>
@@ -19909,11 +19951,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>TailRecovery_UP!B16</f>
+        <f>TailRecovery_UP!B17</f>
         <v/>
       </c>
       <c r="C12">
-        <f>TailRecovery_DOWN!B16</f>
+        <f>TailRecovery_DOWN!B17</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Make workbook LibreOffice-compatible and complete runtime PASS checks
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step.xlsx
@@ -9641,7 +9641,7 @@
         </is>
       </c>
       <c r="B223">
-        <f>IF(B222="N/A",0,XLOOKUP(B222,A7:A206,D7:D206,0))</f>
+        <f>IF(B222="N/A",0,INDEX(D7:D206,MATCH(B222,A7:A206,0)))</f>
         <v/>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
         </is>
       </c>
       <c r="B224">
-        <f>IF(B222="N/A",0,ABS(XLOOKUP(B222,A7:A206,H7:H206,0)))</f>
+        <f>IF(B222="N/A",0,ABS(INDEX(H7:H206,MATCH(B222,A7:A206,0))))</f>
         <v/>
       </c>
     </row>
@@ -18269,7 +18269,7 @@
         </is>
       </c>
       <c r="B223">
-        <f>IF(B222="N/A",0,XLOOKUP(B222,A7:A206,D7:D206,0))</f>
+        <f>IF(B222="N/A",0,INDEX(D7:D206,MATCH(B222,A7:A206,0)))</f>
         <v/>
       </c>
     </row>
@@ -18280,7 +18280,7 @@
         </is>
       </c>
       <c r="B224">
-        <f>IF(B222="N/A",0,ABS(XLOOKUP(B222,A7:A206,H7:H206,0)))</f>
+        <f>IF(B222="N/A",0,ABS(INDEX(H7:H206,MATCH(B222,A7:A206,0))))</f>
         <v/>
       </c>
     </row>
@@ -18306,7 +18306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18360,7 +18360,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>XLOOKUP(B4,Settings!A21:A24,Settings!B21:B24)</f>
+        <f>INDEX(Settings!B21:B24,MATCH(B4,Settings!A21:A24,0))</f>
         <v/>
       </c>
     </row>
@@ -18371,7 +18371,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>XLOOKUP(B4,Settings!A21:A24,Settings!C21:C24)</f>
+        <f>INDEX(Settings!C21:C24,MATCH(B4,Settings!A21:A24,0))</f>
         <v/>
       </c>
     </row>
@@ -18437,7 +18437,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>IF(Scenario_UP!B4&gt;=INDEX(Scenario_UP!E4:E7,B4),"YES","NO")</f>
+        <f>IF(Scenario_UP!B4&gt;=IF(B4=1,Scenario_UP!E4,IF(B4=2,Scenario_UP!E5,IF(B4=3,Scenario_UP!E6,Scenario_UP!E7))),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -18516,15 +18516,40 @@
       </c>
       <c r="K20" s="1" t="inlineStr">
         <is>
+          <t>Lots</t>
+        </is>
+      </c>
+      <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>CostMultiplier</t>
+        </is>
+      </c>
+      <c r="M20" s="1" t="inlineStr">
+        <is>
+          <t>SpreadCost</t>
+        </is>
+      </c>
+      <c r="N20" s="1" t="inlineStr">
+        <is>
+          <t>CommissionCost</t>
+        </is>
+      </c>
+      <c r="O20" s="1" t="inlineStr">
+        <is>
+          <t>SwapCost</t>
+        </is>
+      </c>
+      <c r="P20" s="1" t="inlineStr">
+        <is>
           <t>Costs</t>
         </is>
       </c>
-      <c r="L20" s="1" t="inlineStr">
+      <c r="Q20" s="1" t="inlineStr">
         <is>
           <t>CycleProfit</t>
         </is>
       </c>
-      <c r="M20" s="1" t="inlineStr">
+      <c r="R20" s="1" t="inlineStr">
         <is>
           <t>CanCloseSection</t>
         </is>
@@ -18573,15 +18598,35 @@
         <v/>
       </c>
       <c r="K21">
-        <f>LET(Lots,C21+F21,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C21+F21</f>
         <v/>
       </c>
       <c r="L21">
-        <f>I21+J21-K21</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M21">
-        <f>IF(L21&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K21*L21</f>
+        <v/>
+      </c>
+      <c r="N21">
+        <f>Settings!$B$13*K21*L21</f>
+        <v/>
+      </c>
+      <c r="O21">
+        <f>Settings!$B$14*K21</f>
+        <v/>
+      </c>
+      <c r="P21">
+        <f>M21+N21+O21</f>
+        <v/>
+      </c>
+      <c r="Q21">
+        <f>I21+J21-P21</f>
+        <v/>
+      </c>
+      <c r="R21">
+        <f>IF(Q21&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -18628,15 +18673,35 @@
         <v/>
       </c>
       <c r="K22">
-        <f>LET(Lots,C22+F22,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C22+F22</f>
         <v/>
       </c>
       <c r="L22">
-        <f>I22+J22-K22</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M22">
-        <f>IF(L22&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K22*L22</f>
+        <v/>
+      </c>
+      <c r="N22">
+        <f>Settings!$B$13*K22*L22</f>
+        <v/>
+      </c>
+      <c r="O22">
+        <f>Settings!$B$14*K22</f>
+        <v/>
+      </c>
+      <c r="P22">
+        <f>M22+N22+O22</f>
+        <v/>
+      </c>
+      <c r="Q22">
+        <f>I22+J22-P22</f>
+        <v/>
+      </c>
+      <c r="R22">
+        <f>IF(Q22&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -18683,15 +18748,35 @@
         <v/>
       </c>
       <c r="K23">
-        <f>LET(Lots,C23+F23,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C23+F23</f>
         <v/>
       </c>
       <c r="L23">
-        <f>I23+J23-K23</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M23">
-        <f>IF(L23&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K23*L23</f>
+        <v/>
+      </c>
+      <c r="N23">
+        <f>Settings!$B$13*K23*L23</f>
+        <v/>
+      </c>
+      <c r="O23">
+        <f>Settings!$B$14*K23</f>
+        <v/>
+      </c>
+      <c r="P23">
+        <f>M23+N23+O23</f>
+        <v/>
+      </c>
+      <c r="Q23">
+        <f>I23+J23-P23</f>
+        <v/>
+      </c>
+      <c r="R23">
+        <f>IF(Q23&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -18738,15 +18823,35 @@
         <v/>
       </c>
       <c r="K24">
-        <f>LET(Lots,C24+F24,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C24+F24</f>
         <v/>
       </c>
       <c r="L24">
-        <f>I24+J24-K24</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M24">
-        <f>IF(L24&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K24*L24</f>
+        <v/>
+      </c>
+      <c r="N24">
+        <f>Settings!$B$13*K24*L24</f>
+        <v/>
+      </c>
+      <c r="O24">
+        <f>Settings!$B$14*K24</f>
+        <v/>
+      </c>
+      <c r="P24">
+        <f>M24+N24+O24</f>
+        <v/>
+      </c>
+      <c r="Q24">
+        <f>I24+J24-P24</f>
+        <v/>
+      </c>
+      <c r="R24">
+        <f>IF(Q24&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -18757,7 +18862,7 @@
         </is>
       </c>
       <c r="B30">
-        <f>IFERROR(INDEX(A21:A24,MATCH("YES",M21:M24,0)),"NONE")</f>
+        <f>IFERROR(INDEX(A21:A24,MATCH("YES",R21:R24,0)),"NONE")</f>
         <v/>
       </c>
     </row>
@@ -18768,7 +18873,7 @@
         </is>
       </c>
       <c r="B31">
-        <f>IF(B30="NONE",0,XLOOKUP(B30,A21:A24,L21:L24,0))</f>
+        <f>IF(B30="NONE",0,INDEX(Q21:Q24,MATCH(B30,A21:A24,0)))</f>
         <v/>
       </c>
     </row>
@@ -18838,7 +18943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18892,7 +18997,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>XLOOKUP(B4,Settings!A21:A24,Settings!B21:B24)</f>
+        <f>INDEX(Settings!B21:B24,MATCH(B4,Settings!A21:A24,0))</f>
         <v/>
       </c>
     </row>
@@ -18903,7 +19008,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>XLOOKUP(B4,Settings!A21:A24,Settings!C21:C24)</f>
+        <f>INDEX(Settings!C21:C24,MATCH(B4,Settings!A21:A24,0))</f>
         <v/>
       </c>
     </row>
@@ -18969,7 +19074,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>IF(Scenario_DOWN!B4&lt;=INDEX(Scenario_DOWN!E9:E12,B4),"YES","NO")</f>
+        <f>IF(Scenario_DOWN!B4&lt;=IF(B4=1,Scenario_DOWN!E9,IF(B4=2,Scenario_DOWN!E10,IF(B4=3,Scenario_DOWN!E11,Scenario_DOWN!E12))),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19048,15 +19153,40 @@
       </c>
       <c r="K20" s="1" t="inlineStr">
         <is>
+          <t>Lots</t>
+        </is>
+      </c>
+      <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>CostMultiplier</t>
+        </is>
+      </c>
+      <c r="M20" s="1" t="inlineStr">
+        <is>
+          <t>SpreadCost</t>
+        </is>
+      </c>
+      <c r="N20" s="1" t="inlineStr">
+        <is>
+          <t>CommissionCost</t>
+        </is>
+      </c>
+      <c r="O20" s="1" t="inlineStr">
+        <is>
+          <t>SwapCost</t>
+        </is>
+      </c>
+      <c r="P20" s="1" t="inlineStr">
+        <is>
           <t>Costs</t>
         </is>
       </c>
-      <c r="L20" s="1" t="inlineStr">
+      <c r="Q20" s="1" t="inlineStr">
         <is>
           <t>CycleProfit</t>
         </is>
       </c>
-      <c r="M20" s="1" t="inlineStr">
+      <c r="R20" s="1" t="inlineStr">
         <is>
           <t>CanCloseSection</t>
         </is>
@@ -19105,15 +19235,35 @@
         <v/>
       </c>
       <c r="K21">
-        <f>LET(Lots,C21+F21,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C21+F21</f>
         <v/>
       </c>
       <c r="L21">
-        <f>I21+J21-K21</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M21">
-        <f>IF(L21&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K21*L21</f>
+        <v/>
+      </c>
+      <c r="N21">
+        <f>Settings!$B$13*K21*L21</f>
+        <v/>
+      </c>
+      <c r="O21">
+        <f>Settings!$B$14*K21</f>
+        <v/>
+      </c>
+      <c r="P21">
+        <f>M21+N21+O21</f>
+        <v/>
+      </c>
+      <c r="Q21">
+        <f>I21+J21-P21</f>
+        <v/>
+      </c>
+      <c r="R21">
+        <f>IF(Q21&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19160,15 +19310,35 @@
         <v/>
       </c>
       <c r="K22">
-        <f>LET(Lots,C22+F22,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C22+F22</f>
         <v/>
       </c>
       <c r="L22">
-        <f>I22+J22-K22</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M22">
-        <f>IF(L22&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K22*L22</f>
+        <v/>
+      </c>
+      <c r="N22">
+        <f>Settings!$B$13*K22*L22</f>
+        <v/>
+      </c>
+      <c r="O22">
+        <f>Settings!$B$14*K22</f>
+        <v/>
+      </c>
+      <c r="P22">
+        <f>M22+N22+O22</f>
+        <v/>
+      </c>
+      <c r="Q22">
+        <f>I22+J22-P22</f>
+        <v/>
+      </c>
+      <c r="R22">
+        <f>IF(Q22&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19215,15 +19385,35 @@
         <v/>
       </c>
       <c r="K23">
-        <f>LET(Lots,C23+F23,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C23+F23</f>
         <v/>
       </c>
       <c r="L23">
-        <f>I23+J23-K23</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M23">
-        <f>IF(L23&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K23*L23</f>
+        <v/>
+      </c>
+      <c r="N23">
+        <f>Settings!$B$13*K23*L23</f>
+        <v/>
+      </c>
+      <c r="O23">
+        <f>Settings!$B$14*K23</f>
+        <v/>
+      </c>
+      <c r="P23">
+        <f>M23+N23+O23</f>
+        <v/>
+      </c>
+      <c r="Q23">
+        <f>I23+J23-P23</f>
+        <v/>
+      </c>
+      <c r="R23">
+        <f>IF(Q23&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19270,15 +19460,35 @@
         <v/>
       </c>
       <c r="K24">
-        <f>LET(Lots,C24+F24,Mult,IF(Settings!$B$19="FULL_CYCLE",2,1),SpreadCost,Settings!$B$12*Settings!$B$4*Lots*Mult,CommissionCost,Settings!$B$13*Lots*Mult,SwapCost,Settings!$B$14*Lots,SpreadCost+CommissionCost+SwapCost)</f>
+        <f>C24+F24</f>
         <v/>
       </c>
       <c r="L24">
-        <f>I24+J24-K24</f>
+        <f>IF(Settings!$B$19="FULL_CYCLE",2,1)</f>
         <v/>
       </c>
       <c r="M24">
-        <f>IF(L24&gt;0,"YES","NO")</f>
+        <f>Settings!$B$12*Settings!$B$4*K24*L24</f>
+        <v/>
+      </c>
+      <c r="N24">
+        <f>Settings!$B$13*K24*L24</f>
+        <v/>
+      </c>
+      <c r="O24">
+        <f>Settings!$B$14*K24</f>
+        <v/>
+      </c>
+      <c r="P24">
+        <f>M24+N24+O24</f>
+        <v/>
+      </c>
+      <c r="Q24">
+        <f>I24+J24-P24</f>
+        <v/>
+      </c>
+      <c r="R24">
+        <f>IF(Q24&gt;0,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19289,7 +19499,7 @@
         </is>
       </c>
       <c r="B30">
-        <f>IFERROR(INDEX(A21:A24,MATCH("YES",M21:M24,0)),"NONE")</f>
+        <f>IFERROR(INDEX(A21:A24,MATCH("YES",R21:R24,0)),"NONE")</f>
         <v/>
       </c>
     </row>
@@ -19300,7 +19510,7 @@
         </is>
       </c>
       <c r="B31">
-        <f>IF(B30="NONE",0,XLOOKUP(B30,A21:A24,L21:L24,0))</f>
+        <f>IF(B30="NONE",0,INDEX(Q21:Q24,MATCH(B30,A21:A24,0)))</f>
         <v/>
       </c>
     </row>
@@ -19546,7 +19756,7 @@
         </is>
       </c>
       <c r="B16">
-        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!B21:B24),Settings!$B$7)</f>
+        <f>FLOOR(B14*INDEX(Settings!B21:B24,MATCH(B15,Settings!A21:A24,0)),Settings!$B$7)</f>
         <v/>
       </c>
     </row>
@@ -19557,7 +19767,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!C21:C24),Settings!$B$7)</f>
+        <f>FLOOR(B14*INDEX(Settings!C21:C24,MATCH(B15,Settings!A21:A24,0)),Settings!$B$7)</f>
         <v/>
       </c>
     </row>
@@ -19748,7 +19958,7 @@
         </is>
       </c>
       <c r="B16">
-        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!B21:B24),Settings!$B$7)</f>
+        <f>FLOOR(B14*INDEX(Settings!B21:B24,MATCH(B15,Settings!A21:A24,0)),Settings!$B$7)</f>
         <v/>
       </c>
     </row>
@@ -19759,7 +19969,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>FLOOR(B14*XLOOKUP(B15,Settings!A21:A24,Settings!C21:C24),Settings!$B$7)</f>
+        <f>FLOOR(B14*INDEX(Settings!C21:C24,MATCH(B15,Settings!A21:A24,0)),Settings!$B$7)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add concrete runtime tail tie-case proof for UP/DOWN checks
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step.xlsx
@@ -9619,7 +9619,7 @@
         </is>
       </c>
       <c r="B221">
-        <f>MINIFS(H7:H206,B7:B206,"SELL",H7:H206,"&lt;0")</f>
+        <f>IFERROR(MIN(IF((B7:B206="SELL")*(H7:H206&lt;0),H7:H206)),0)</f>
         <v/>
       </c>
     </row>
@@ -9630,7 +9630,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IFERROR(MINIFS(A7:A206,B7:B206,"SELL",H7:H206,B221),"N/A")</f>
+        <f>IFERROR(MIN(IF((B7:B206="SELL")*(H7:H206=B221),A7:A206)),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -18247,7 +18247,7 @@
         </is>
       </c>
       <c r="B221">
-        <f>MINIFS(H7:H206,B7:B206,"BUY",H7:H206,"&lt;0")</f>
+        <f>IFERROR(MIN(IF((B7:B206="BUY")*(H7:H206&lt;0),H7:H206)),0)</f>
         <v/>
       </c>
     </row>
@@ -18258,7 +18258,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IFERROR(MINIFS(A7:A206,B7:B206,"BUY",H7:H206,B221),"N/A")</f>
+        <f>IFERROR(MIN(IF((B7:B206="BUY")*(H7:H206=B221),A7:A206)),"N/A")</f>
         <v/>
       </c>
     </row>

</xml_diff>